<commit_message>
v1.6-results: E9 second domain (cloud/API capacity, D44): supply domain proven byte-identical to v1.4.1-results; 84 scripted runs; refreshed NUMBERS.md (RQ5), tables, workbook, paper pack; every prior number identical to v1.5-results
</commit_message>
<xml_diff>
--- a/paper_pack/results_all.xlsx
+++ b/paper_pack/results_all.xlsx
@@ -22,7 +22,8 @@
     <sheet name="reputation grid" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Enron" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="E8" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="TLA+ verification" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="E9" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="TLA+ verification" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,13 +433,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E325"/>
+  <dimension ref="A1:E342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Outcome-Bound Trust: all results (tag v1.5-results). Built from results/ and spec/results/ only by `python -m eval.pack`; numbers are as printed in the paper tables and NUMBERS.md.</t>
+          <t>Outcome-Bound Trust: all results (tag v1.6-results). Built from results/ and spec/results/ only by `python -m eval.pack`; numbers are as printed in the paper tables and NUMBERS.md.</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1600,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1978,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2383,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2950,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3517,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
@@ -4353,7 +4354,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
@@ -4731,7 +4732,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
@@ -5730,7 +5731,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
@@ -6081,7 +6082,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6433,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
@@ -8167,459 +8168,459 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9, second domain (an agent buying cloud/API capacity; scripted buyer and provid</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>defense (OBT variants, reputation variants, baselines)</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9, second domain (an agent buying cloud/API capacity; scripted buyer and provid</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>seeds</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>seeds in the mean</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9, second domain (an agent buying cloud/API capacity; scripted buyer and provid</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>loss from lies</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>mean over attack scenarios 2-12 of cost − cost of the honest run (same defense, seed), $ per run; [95% bootstrap CI over seeds] where shown</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9, second domain (an agent buying cloud/API capacity; scripted buyer and provid</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>cost against the same decisions with every relied-on promise kept (DESIGN §6), $</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9, second domain (an agent buying cloud/API capacity; scripted buyer and provid</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>reroute premium</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>backup premium on quantity rerouted after the defense's own blocks, differenced vs the honest run, $ per run</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9, second domain (an agent buying cloud/API capacity; scripted buyer and provid</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>resid</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>loss from lies − damage − reroute premium, $ per run</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9, second domain (an agent buying cloud/API capacity; scripted buyer and provid</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>utility cost</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>cost(defense) − cost(none) on the honest scenario, same seed, $ per run</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9, second domain (an agent buying cloud/API capacity; scripted buyer and provid</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>utility (% of cost)</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>utility cost as a % of the honest run's total cost without a defense</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9, second domain (an agent buying cloud/API capacity; scripted buyer and provid</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>provider share</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>share of reserved capacity units bought from the main provider, honest scenario (E9)</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 damage against the per-event bound (OBT runs; QUOTA and SLA events; docs/E9_P</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_damage_vs_bound</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>events</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>failure-event type (QUOTA, SLA, all)</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 damage against the per-event bound (OBT runs; QUOTA and SLA events; docs/E9_P</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_damage_vs_bound</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>failure events</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>FAILED claims with consumed units</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 damage against the per-event bound (OBT runs; QUOTA and SLA events; docs/E9_P</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_damage_vs_bound</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>runs with events</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>OBT runs with at least one event</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 damage against the per-event bound (OBT runs; QUOTA and SLA events; docs/E9_P</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_damage_vs_bound</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>sum of bounds</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>sum of per-event bounds Σ L_e, $</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 damage against the per-event bound (OBT runs; QUOTA and SLA events; docs/E9_P</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_damage_vs_bound</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>cost against the same decisions with every relied-on promise kept (DESIGN §6), $</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 damage against the per-event bound (OBT runs; QUOTA and SLA events; docs/E9_P</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_damage_vs_bound</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>max damage/bound</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>largest per-run damage / Σ L_e</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 damage against the per-event bound (OBT runs; QUOTA and SLA events; docs/E9_P</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_damage_vs_bound</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>max damage/a-priori</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>largest damage / k-scaled a-priori bound</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 damage against the per-event bound (OBT runs; QUOTA and SLA events; docs/E9_P</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_damage_vs_bound</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>held</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>damage ≤ Σ L_e in every run</t>
         </is>
       </c>
     </row>
@@ -8631,22 +8632,22 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>mutant</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>guard removed in the spec (none = unmutated)</t>
         </is>
       </c>
     </row>
@@ -8658,22 +8659,22 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>verdict</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
         </is>
       </c>
     </row>
@@ -8685,22 +8686,22 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>violation</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>property TLC reported violated</t>
         </is>
       </c>
     </row>
@@ -8712,22 +8713,22 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>distinct_states</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>distinct states when TLC stopped</t>
         </is>
       </c>
     </row>
@@ -8739,22 +8740,22 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>depth</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
         </is>
       </c>
     </row>
@@ -8766,22 +8767,22 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>runtime_s</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
         </is>
       </c>
     </row>
@@ -8793,22 +8794,22 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>mutant</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>guard removed in the spec (none = unmutated)</t>
         </is>
       </c>
     </row>
@@ -8820,22 +8821,22 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>verdict</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
         </is>
       </c>
     </row>
@@ -8847,22 +8848,22 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>violation</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>property TLC reported violated</t>
         </is>
       </c>
     </row>
@@ -8874,22 +8875,22 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>distinct_states</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>distinct states when TLC stopped</t>
         </is>
       </c>
     </row>
@@ -8901,22 +8902,22 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>depth</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
         </is>
       </c>
     </row>
@@ -8928,22 +8929,22 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>runtime_s</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
         </is>
       </c>
     </row>
@@ -8955,22 +8956,22 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/fallbackB_summary.txt</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>mutant</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>guard removed in the spec (none = unmutated)</t>
         </is>
       </c>
     </row>
@@ -8982,22 +8983,22 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackB_summary.txt</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>verdict</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
         </is>
       </c>
     </row>
@@ -9009,22 +9010,22 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackB_summary.txt</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>violation</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>property TLC reported violated</t>
         </is>
       </c>
     </row>
@@ -9036,22 +9037,22 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackB_summary.txt</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>quick</t>
+          <t>distinct_states</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>distinct states when TLC stopped</t>
         </is>
       </c>
     </row>
@@ -9063,22 +9064,22 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackB_summary.txt</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>A'</t>
+          <t>depth</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
         </is>
       </c>
     </row>
@@ -9090,22 +9091,22 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackB_summary.txt</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>runtime_s</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
         </is>
       </c>
     </row>
@@ -9117,22 +9118,22 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/quick_b01_summary.txt</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>quick B0=1</t>
+          <t>mutant</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>guard removed in the spec (none = unmutated)</t>
         </is>
       </c>
     </row>
@@ -9144,20 +9145,479 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>property TLC reported violated</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>distinct_states</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>distinct states when TLC stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>runtime_s</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>guard removed in the spec (none = unmutated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>property TLC reported violated</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>distinct_states</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>distinct states when TLC stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>runtime_s</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
           <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
         </is>
       </c>
-      <c r="C325" t="inlineStr">
+      <c r="C336" t="inlineStr">
         <is>
           <t>spec/results/k_coverage.txt</t>
         </is>
       </c>
-      <c r="D325" t="inlineStr">
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>guard removed in the spec (none = unmutated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>covered</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>quick</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>A'</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>quick B0=1</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
         <is>
           <t>A' B0=1</t>
         </is>
       </c>
-      <c r="E325" t="inlineStr">
+      <c r="E342" t="inlineStr">
         <is>
           <t>as in the source file</t>
         </is>
@@ -17677,6 +18137,386 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>E9, second domain (an agent buying cloud/API capacity; scripted buyer and providers, structured intents, no natural-language extraction; seeds 1-3): loss from lies (mean of scenarios 2-7) and utility cost against none, mean [95% bootstrap CI over seeds]; damage + reroute premium + resid are means over attack runs; $ per run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>source: results/tables.json → e9</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>defense</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>seeds</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>loss from lies</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>reroute premium</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>resid</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>utility cost</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>utility (% of cost)</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>provider share</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1,165.9 [1,120.7, 1,197.8]</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1165.9</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.0 [0.0, 0.0]</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.974</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>134.9 [116.0, 145.0]</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>134.9</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>266.0 [240.0, 304.0]</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>18.34</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.193</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>rep-n18</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>477.2 [437.8, 512.7]</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>477.2</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.0 [0.0, 0.0]</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.974</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>42.6 [34.8, 53.2]</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>327.3 [310.0, 346.0]</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>22.57</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.111</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>E9 damage against the per-event bound (OBT runs; QUOTA and SLA events; docs/E9_PLAN.md §4). A ratio above 1 would break the bound.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>source: results/tables.json → e9_damage_vs_bound</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>events</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>failure events</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>runs with events</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>sum of bounds</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>max damage/bound</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>max damage/a-priori</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>held</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>QUOTA</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>54</v>
+      </c>
+      <c r="C12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" t="n">
+        <v>910</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SLA</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>41</v>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" t="n">
+        <v>342</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>95</v>
+      </c>
+      <c r="C14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1252</v>
+      </c>
+      <c r="E14" t="n">
+        <v>366</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
v1.7-results: E9 calibration (D45): OBT b0 x k and reputation D33 grid on the cloud domain, configs chosen by E1's rule; transferred vs calibrated side by side, Pareto fronts, bound held in all 168 OBT grid runs; legacy summary key renamed (no 'price of safety' anywhere); every prior number identical to v1.6-results
</commit_message>
<xml_diff>
--- a/paper_pack/results_all.xlsx
+++ b/paper_pack/results_all.xlsx
@@ -23,7 +23,8 @@
     <sheet name="Enron" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="E8" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="E9" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="TLA+ verification" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="E9 calibration" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="TLA+ verification" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,13 +434,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E342"/>
+  <dimension ref="A1:E368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Outcome-Bound Trust: all results (tag v1.6-results). Built from results/ and spec/results/ only by `python -m eval.pack`; numbers are as printed in the paper tables and NUMBERS.md.</t>
+          <t>Outcome-Bound Trust: all results (tag v1.7-results). Built from results/ and spec/results/ only by `python -m eval.pack`; numbers are as printed in the paper tables and NUMBERS.md.</t>
         </is>
       </c>
     </row>
@@ -493,7 +494,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OBT config: b0 fraction, window W, grace δ</t>
+          <t>config: E1, OBT b0 fraction, window W, grace δ; E9 calibration, grid point and its settings</t>
         </is>
       </c>
     </row>
@@ -601,7 +602,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>OBT config: b0 fraction, window W, grace δ</t>
+          <t>config: E1, OBT b0 fraction, window W, grace δ; E9 calibration, grid point and its settings</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6785,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>the chosen reputation config (D33)</t>
+          <t>the config chosen by the selection rule (D33 reputation grid; D45 E9 calibration)</t>
         </is>
       </c>
     </row>
@@ -8627,702 +8628,702 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t xml:space="preserve">E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain </t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>defense (OBT variants, reputation variants, baselines)</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t xml:space="preserve">E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain </t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>E9 config source: transferred from the supply domain (D44) or calibrated on the cloud domain (D45)</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t xml:space="preserve">E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain </t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>config</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>config: E1, OBT b0 fraction, window W, grace δ; E9 calibration, grid point and its settings</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t xml:space="preserve">E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain </t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>loss from lies</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>mean over attack scenarios 2-12 of cost − cost of the honest run (same defense, seed), $ per run; [95% bootstrap CI over seeds] where shown</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t xml:space="preserve">E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain </t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>cost against the same decisions with every relied-on promise kept (DESIGN §6), $</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t xml:space="preserve">E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain </t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>reroute premium</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>backup premium on quantity rerouted after the defense's own blocks, differenced vs the honest run, $ per run</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t xml:space="preserve">E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain </t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>resid</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>loss from lies − damage − reroute premium, $ per run</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t xml:space="preserve">E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain </t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>utility cost</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>cost(defense) − cost(none) on the honest scenario, same seed, $ per run</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t xml:space="preserve">E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain </t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>utility (% of cost)</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>utility cost as a % of the honest run's total cost without a defense</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t xml:space="preserve">E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain </t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>provider share</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>share of reserved capacity units bought from the main provider, honest scenario (E9)</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 calibration (D45): the loss bound over every OBT grid run (8 points x 7 scena</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration_bound</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>OBT runs</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>OBT grid runs checked</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 calibration (D45): the loss bound over every OBT grid run (8 points x 7 scena</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration_bound</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>failure events</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>FAILED claims with consumed units</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 calibration (D45): the loss bound over every OBT grid run (8 points x 7 scena</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_bound</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>max damage/bound</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>largest per-run damage / Σ L_e</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 calibration (D45): the loss bound over every OBT grid run (8 points x 7 scena</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_bound</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>held</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>damage ≤ Σ L_e in every run</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 calibration (D45): the loss bound over every OBT grid run (8 points x 7 scena</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_bound</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>invariant violations</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>invariant violations over every grid run (target 0)</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 calibration (D45): the loss bound over every OBT grid run (8 points x 7 scena</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_bound</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>transferred points reproduce E9</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>the transferred grid points' costs equal E9's runs exactly</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. O</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_grid</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>defense (OBT variants, reputation variants, baselines)</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. O</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_grid</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>point</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>E9 calibration grid point</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. O</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_grid</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>utility cost</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>cost(defense) − cost(none) on the honest scenario, same seed, $ per run</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. O</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_grid</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>loss from lies</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>mean over attack scenarios 2-12 of cost − cost of the honest run (same defense, seed), $ per run; [95% bootstrap CI over seeds] where shown</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. O</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_grid</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>never trades</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>never trades with an honest S_main</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. O</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_grid</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>locks out</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>never trades after a lock-out</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. O</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_grid</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>front</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>on the defense's Pareto front (never-trading points excluded)</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. O</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_grid</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>chosen</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>the config chosen by the selection rule (D33 reputation grid; D45 E9 calibration)</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. O</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_grid</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>transferred</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>the config E9 ran with (D44)</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. O</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_grid</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>max damage/bound</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>largest per-run damage / Σ L_e</t>
         </is>
       </c>
     </row>
@@ -9334,22 +9335,22 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>mutant</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>guard removed in the spec (none = unmutated)</t>
         </is>
       </c>
     </row>
@@ -9361,22 +9362,22 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>verdict</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
         </is>
       </c>
     </row>
@@ -9388,22 +9389,22 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>violation</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>property TLC reported violated</t>
         </is>
       </c>
     </row>
@@ -9415,22 +9416,22 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>distinct_states</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>distinct states when TLC stopped</t>
         </is>
       </c>
     </row>
@@ -9442,22 +9443,22 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>depth</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
         </is>
       </c>
     </row>
@@ -9469,22 +9470,22 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>runtime_s</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
         </is>
       </c>
     </row>
@@ -9496,22 +9497,22 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>quick</t>
+          <t>mutant</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>guard removed in the spec (none = unmutated)</t>
         </is>
       </c>
     </row>
@@ -9523,22 +9524,22 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>A'</t>
+          <t>verdict</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
         </is>
       </c>
     </row>
@@ -9550,22 +9551,22 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>violation</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>property TLC reported violated</t>
         </is>
       </c>
     </row>
@@ -9577,22 +9578,22 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>quick B0=1</t>
+          <t>distinct_states</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>distinct states when TLC stopped</t>
         </is>
       </c>
     </row>
@@ -9604,20 +9605,722 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_summary.txt</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_summary.txt</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>runtime_s</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>guard removed in the spec (none = unmutated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>property TLC reported violated</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>distinct_states</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>distinct states when TLC stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>runtime_s</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>guard removed in the spec (none = unmutated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>property TLC reported violated</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>distinct_states</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>distinct states when TLC stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>runtime_s</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>guard removed in the spec (none = unmutated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>property TLC reported violated</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>distinct_states</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>distinct states when TLC stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>runtime_s</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
           <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
+      <c r="C362" t="inlineStr">
         <is>
           <t>spec/results/k_coverage.txt</t>
         </is>
       </c>
-      <c r="D342" t="inlineStr">
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>guard removed in the spec (none = unmutated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>covered</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>quick</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>A'</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>quick B0=1</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
         <is>
           <t>A' B0=1</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr">
+      <c r="E368" t="inlineStr">
         <is>
           <t>as in the source file</t>
         </is>
@@ -18517,6 +19220,1474 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>E9 with transferred vs calibrated configs (D45). Transferred: the supply-domain configs E9 ran with (D44). Calibrated: each defense's cloud-domain grid point chosen by E1's rule (Pareto front in utility cost and attack loss, smallest sum; never-trading points excluded). Seeds 1-3, mean [95% bootstrap CI over seeds]; $ per run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>source: results/tables.json → e9_calibration</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>defense</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>loss from lies</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>reroute premium</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>resid</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>utility cost</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>utility (% of cost)</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>provider share</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>obt_b0.05_k1 (b0_frac 0.05, budget_k 1)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>42.6 [34.8, 53.2]</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>327.3 [310.0, 346.0]</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>22.57</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.111</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>calibrated</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>obt_b0.2_k1 (b0_frac 0.2, budget_k 1)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>46.3 [40.8, 50.0]</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="F5" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-57.8</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>293.7 [269.0, 323.0]</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.222</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>rep_n3_th0.9_cap200 (rep_n0 3, rep_theta 0.9, rep_cap 200.0)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>134.9 [116.0, 145.0]</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>134.9</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>266.0 [240.0, 304.0]</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>18.34</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.193</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>calibrated</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>rep_n8_th0.8_cap200 (rep_n0 8, rep_theta 0.8, rep_cap 200.0)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>371.0 [340.8, 387.0]</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>371</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.0 [0.0, 0.0]</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.974</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>E9 calibration (D45): the loss bound over every OBT grid run (8 points x 7 scenarios x 3 seeds), and the harness check that the transferred grid points reproduce E9's runs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>source: results/tables.json → e9_calibration_bound</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>OBT runs</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>failure events</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>max damage/bound</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>held</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>invariant violations</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>transferred points reproduce E9</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="n"/>
+      <c r="H11" s="1" t="n"/>
+      <c r="I11" s="1" t="n"/>
+      <c r="J11" s="1" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>168</v>
+      </c>
+      <c r="B12" t="n">
+        <v>586</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>E9 calibration grids (D45): every point, scripted buyer, seeds 1-3, $ per run. OBT over b0 (fraction of per-round spend) and k; reputation over n0, theta and cap (the D33 grid). Max damage/bound over the point's OBT runs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>source: results/tables.json → e9_calibration_grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>defense</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>point</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>utility cost</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>loss from lies</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>never trades</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>locks out</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>front</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>chosen</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="J16" s="1" t="inlineStr">
+        <is>
+          <t>max damage/bound</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>obt_b0.025_k1</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>obt_b0.025_k2</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>obt_b0.05_k1</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>327.3</v>
+      </c>
+      <c r="D19" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>obt_b0.05_k2</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>303.7</v>
+      </c>
+      <c r="D20" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>0.423</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>obt_b0.1_k1</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>284.7</v>
+      </c>
+      <c r="D21" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>obt_b0.1_k2</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>246.7</v>
+      </c>
+      <c r="D22" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>obt_b0.2_k1</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>293.7</v>
+      </c>
+      <c r="D23" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="n">
+        <v>0.411</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>obt_b0.2_k2</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>244.7</v>
+      </c>
+      <c r="D24" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="n">
+        <v>0.8149999999999999</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>rep_n3_th0.8_cap100</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>rep_n3_th0.8_cap200</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>405.8</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>rep_n3_th0.8_cap400</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>482</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>rep_n3_th0.85_cap100</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>rep_n3_th0.85_cap200</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>266</v>
+      </c>
+      <c r="D29" t="n">
+        <v>134.9</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>rep_n3_th0.85_cap400</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>266</v>
+      </c>
+      <c r="D30" t="n">
+        <v>211.1</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>rep_n3_th0.9_cap100</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>rep_n3_th0.9_cap200</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>266</v>
+      </c>
+      <c r="D32" t="n">
+        <v>134.9</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>rep_n3_th0.9_cap400</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>266</v>
+      </c>
+      <c r="D33" t="n">
+        <v>211.1</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>rep_n8_th0.8_cap100</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>rep_n8_th0.8_cap200</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>371</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>rep_n8_th0.8_cap400</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>475.4</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>rep_n8_th0.85_cap100</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>rep_n8_th0.85_cap200</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>384.7</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>rep_n8_th0.85_cap400</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>489.1</v>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>rep_n8_th0.9_cap100</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>rep_n8_th0.9_cap200</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>384.7</v>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>rep_n8_th0.9_cap400</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>489.1</v>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>rep_n18_th0.8_cap100</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>rep_n18_th0.8_cap200</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>476.8</v>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>rep_n18_th0.8_cap400</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>641.2</v>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>rep_n18_th0.85_cap100</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>rep_n18_th0.85_cap200</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>476.8</v>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>rep_n18_th0.85_cap400</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>641.2</v>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>rep_n18_th0.9_cap100</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>rep_n18_th0.9_cap200</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" t="n">
+        <v>477.2</v>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>rep-strict</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>rep_n18_th0.9_cap400</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" t="n">
+        <v>641.6</v>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
v1.8-results: E9 extended OBT calibration grid (D45a): 18 points, pick unchanged (b0 20%, k 1; on the k = 1 lower limit, not extended further); bound held in all 378 runs; every prior number identical to v1.7-results
</commit_message>
<xml_diff>
--- a/paper_pack/results_all.xlsx
+++ b/paper_pack/results_all.xlsx
@@ -24,7 +24,8 @@
     <sheet name="E8" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="E9" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="E9 calibration" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="TLA+ verification" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="E9 calibration ext" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="TLA+ verification" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,13 +435,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E368"/>
+  <dimension ref="A1:E395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Outcome-Bound Trust: all results (tag v1.7-results). Built from results/ and spec/results/ only by `python -m eval.pack`; numbers are as printed in the paper tables and NUMBERS.md.</t>
+          <t>Outcome-Bound Trust: all results (tag v1.8-results). Built from results/ and spec/results/ only by `python -m eval.pack`; numbers are as printed in the paper tables and NUMBERS.md.</t>
         </is>
       </c>
     </row>
@@ -9330,729 +9331,729 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>defense (OBT variants, reputation variants, baselines)</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>E9 config source: transferred from the supply domain (D44) or calibrated on the cloud domain (D45)</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>config</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>config: E1, OBT b0 fraction, window W, grace δ; E9 calibration, grid point and its settings</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>loss from lies</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>mean over attack scenarios 2-12 of cost − cost of the honest run (same defense, seed), $ per run; [95% bootstrap CI over seeds] where shown</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>cost against the same decisions with every relied-on promise kept (DESIGN §6), $</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>spec/results/quick_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>reroute premium</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>backup premium on quantity rerouted after the defense's own blocks, differenced vs the honest run, $ per run</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>resid</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>loss from lies − damage − reroute premium, $ per run</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>utility cost</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>cost(defense) − cost(none) on the honest scenario, same seed, $ per run</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>utility (% of cost)</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>utility cost as a % of the honest run's total cost without a defense</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>provider share</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>share of reserved capacity units bought from the main provider, honest scenario (E9)</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 extended OBT grid (D45a): the loss bound over every run (18 points x 7 scenar</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_bound</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>OBT runs</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>OBT grid runs checked</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+          <t>E9 extended OBT grid (D45a): the loss bound over every run (18 points x 7 scenar</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_bound</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>failure events</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>FAILED claims with consumed units</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 extended OBT grid (D45a): the loss bound over every run (18 points x 7 scenar</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_bound</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>max damage/bound</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>largest per-run damage / Σ L_e</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 extended OBT grid (D45a): the loss bound over every run (18 points x 7 scenar</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_bound</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>held</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>damage ≤ Σ L_e in every run</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 extended OBT grid (D45a): the loss bound over every run (18 points x 7 scenar</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_bound</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>invariant violations</t>
         </is>
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>invariant violations over every grid run (target 0)</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 extended OBT grid (D45a): the loss bound over every run (18 points x 7 scenar</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_bound</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>pick moved</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>the rule's OBT pick differs from D45's</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t>E9 extended OBT grid (D45a): the loss bound over every run (18 points x 7 scenar</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_bound</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>pick on grid edge</t>
         </is>
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>edges of the extended grid the OBT pick sits on (b0/k min or max)</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+          <t xml:space="preserve">E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. </t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>spec/results/fallbackB_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_grid</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>point</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>E9 calibration grid point</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. </t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_grid</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>b0</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>OBT b0 as a fraction of expected per-round spend</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. </t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_grid</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>k</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>budget growth multiplier (D36)</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. </t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_grid</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>utility cost</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>cost(defense) − cost(none) on the honest scenario, same seed, $ per run</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. </t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_grid</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>loss from lies</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>mean over attack scenarios 2-12 of cost − cost of the honest run (same defense, seed), $ per run; [95% bootstrap CI over seeds] where shown</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. </t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_grid</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>never trades</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>never trades with an honest S_main</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+          <t xml:space="preserve">E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. </t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>spec/results/quick_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_grid</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>front</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>on the defense's Pareto front (never-trading points excluded)</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. </t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_grid</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>chosen</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>the config chosen by the selection rule (D33 reputation grid; D45 E9 calibration)</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. </t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_grid</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>new in D45a</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+          <t>grid point added by the D45a extension</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>TLA+ verification</t>
+          <t>E9 calibration ext</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. </t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>results/tables.json → e9_calibration_ext_grid</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>violation</t>
+          <t>max damage/bound</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>property TLC reported violated</t>
+          <t>largest per-run damage / Σ L_e</t>
         </is>
       </c>
     </row>
@@ -10064,22 +10065,22 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>distinct_states</t>
+          <t>mutant</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>distinct states when TLC stopped</t>
+          <t>guard removed in the spec (none = unmutated)</t>
         </is>
       </c>
     </row>
@@ -10091,22 +10092,22 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>depth</t>
+          <t>verdict</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
         </is>
       </c>
     </row>
@@ -10118,22 +10119,22 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>spec/results/fallbackA2_b01_summary.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>runtime_s</t>
+          <t>violation</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>wall-clock seconds (B: not reported, host sleep)</t>
+          <t>property TLC reported violated</t>
         </is>
       </c>
     </row>
@@ -10145,22 +10146,22 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>mutant</t>
+          <t>distinct_states</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>guard removed in the spec (none = unmutated)</t>
+          <t>distinct states when TLC stopped</t>
         </is>
       </c>
     </row>
@@ -10172,22 +10173,22 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>depth</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
         </is>
       </c>
     </row>
@@ -10199,22 +10200,22 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t xml:space="preserve">TLA+ k = 1, quick: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders = {o1, </t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/quick_summary.txt</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>quick</t>
+          <t>runtime_s</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
         </is>
       </c>
     </row>
@@ -10226,22 +10227,22 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>A'</t>
+          <t>mutant</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>guard removed in the spec (none = unmutated)</t>
         </is>
       </c>
     </row>
@@ -10253,22 +10254,22 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>verdict</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
         </is>
       </c>
     </row>
@@ -10280,22 +10281,22 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>spec/results/k_coverage.txt</t>
+          <t>spec/results/fallbackA2_summary.txt</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>quick B0=1</t>
+          <t>violation</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>as in the source file</t>
+          <t>property TLC reported violated</t>
         </is>
       </c>
     </row>
@@ -10307,20 +10308,749 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_summary.txt</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>distinct_states</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>distinct states when TLC stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_summary.txt</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Orders = {o1,</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_summary.txt</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>runtime_s</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>guard removed in the spec (none = unmutated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>property TLC reported violated</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>distinct_states</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>distinct states when TLC stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLA+ k = 1, B: Sups = {s1} Items = {i1, i2} Claims = {k1, k2, k3} Orders = {o1, </t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackB_summary.txt</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>runtime_s</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>guard removed in the spec (none = unmutated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>property TLC reported violated</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>distinct_states</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>distinct states when TLC stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, quick, B0 = 1: Sups = {s1} Items = {i1} Claims = {k1, k2, k3} Orders</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>spec/results/quick_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>runtime_s</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>guard removed in the spec (none = unmutated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>TLC result: PASS, CAUGHT(property) or N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>property TLC reported violated</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>distinct_states</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>distinct states when TLC stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>depth</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>search depth (PASS) or counterexample length (CAUGHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1, A′, B0 = 1: Sups = {s1, s2} Items = {i1} Claims = {k1, k2, k3} Order</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>spec/results/fallbackA2_b01_summary.txt</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>runtime_s</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>wall-clock seconds (B: not reported, host sleep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
           <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
         </is>
       </c>
-      <c r="C368" t="inlineStr">
+      <c r="C389" t="inlineStr">
         <is>
           <t>spec/results/k_coverage.txt</t>
         </is>
       </c>
-      <c r="D368" t="inlineStr">
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>mutant</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>guard removed in the spec (none = unmutated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>covered</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>quick</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>A'</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>quick B0=1</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>as in the source file</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>TLA+ verification</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>TLA+ k = 1 mutant coverage (every mutant caught in ≥ 1 config)</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>spec/results/k_coverage.txt</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
         <is>
           <t>A' B0=1</t>
         </is>
       </c>
-      <c r="E368" t="inlineStr">
+      <c r="E395" t="inlineStr">
         <is>
           <t>as in the source file</t>
         </is>
@@ -20688,6 +21418,923 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>E9 OBT calibration on the extended grid (D45a: b0 2.5-80% of per-round spend x k 1, 2, 4), same rule as D45, next to the transferred config and D45's pick. Seeds 1-3, mean [95% bootstrap CI over seeds]; $ per run. Pick moved: no; pick on a grid edge: k min.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>source: results/tables.json → e9_calibration_ext</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>defense</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>loss from lies</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>reroute premium</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>resid</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>utility cost</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>utility (% of cost)</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>provider share</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>obt_b0.05_k1 (b0_frac 0.05, budget_k 1)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>42.6 [34.8, 53.2]</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>327.3 [310.0, 346.0]</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>22.57</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.111</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>calibrated, D45 grid</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>obt_b0.2_k1 (b0_frac 0.2, budget_k 1)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>46.3 [40.8, 50.0]</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="F5" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-57.8</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>293.7 [269.0, 323.0]</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.222</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>obt</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>calibrated, extended grid</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>obt_b0.2_k1 (b0_frac 0.2, budget_k 1)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>46.3 [40.8, 50.0]</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-57.8</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>293.7 [269.0, 323.0]</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.222</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>E9 extended OBT grid (D45a): the loss bound over every run (18 points x 7 scenarios x 3 seeds).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>source: results/tables.json → e9_calibration_ext_bound</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>OBT runs</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>failure events</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>max damage/bound</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>held</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>invariant violations</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>pick moved</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>pick on grid edge</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="n"/>
+      <c r="I10" s="1" t="n"/>
+      <c r="J10" s="1" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>378</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>k min</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>E9 extended OBT grid (D45a): every point, scripted buyer, seeds 1-3, $ per run. Max damage/bound over the point's runs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>source: results/tables.json → e9_calibration_ext_grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>point</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>b0</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>utility cost</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>loss from lies</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>never trades</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>front</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>chosen</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>new in D45a</t>
+        </is>
+      </c>
+      <c r="J15" s="1" t="inlineStr">
+        <is>
+          <t>max damage/bound</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>obt_b0.025_k1</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>obt_b0.025_k2</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>obt_b0.025_k4</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" t="n">
+        <v>413.7</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>obt_b0.05_k1</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>327.3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>obt_b0.05_k2</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>303.7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>0.423</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>obt_b0.05_k4</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" t="n">
+        <v>254.7</v>
+      </c>
+      <c r="E21" t="n">
+        <v>112.7</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>0.8149999999999999</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>obt_b0.1_k1</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>284.7</v>
+      </c>
+      <c r="E22" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>obt_b0.1_k2</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>246.7</v>
+      </c>
+      <c r="E23" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>obt_b0.1_k4</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>248.7</v>
+      </c>
+      <c r="E24" t="n">
+        <v>112.1</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>0.8149999999999999</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>obt_b0.2_k1</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>293.7</v>
+      </c>
+      <c r="E25" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="n">
+        <v>0.411</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>obt_b0.2_k2</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>244.7</v>
+      </c>
+      <c r="E26" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="n">
+        <v>0.8149999999999999</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>obt_b0.2_k4</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" t="n">
+        <v>251.3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>116</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>0.8149999999999999</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>obt_b0.4_k1</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>247.3</v>
+      </c>
+      <c r="E28" t="n">
+        <v>146.1</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>0.792</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>obt_b0.4_k2</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" t="n">
+        <v>186.3</v>
+      </c>
+      <c r="E29" t="n">
+        <v>187.7</v>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>obt_b0.4_k4</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C30" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" t="n">
+        <v>186.3</v>
+      </c>
+      <c r="E30" t="n">
+        <v>188.7</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>obt_b0.8_k1</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>183</v>
+      </c>
+      <c r="E31" t="n">
+        <v>275.9</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>0.898</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>obt_b0.8_k2</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" t="n">
+        <v>183</v>
+      </c>
+      <c r="E32" t="n">
+        <v>275.9</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>0.898</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>obt_b0.8_k4</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="n">
+        <v>183</v>
+      </c>
+      <c r="E33" t="n">
+        <v>277.6</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>0.898</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>